<commit_message>
record provisional exclusion preference for MAIN-0076
</commit_message>
<xml_diff>
--- a/系统评价_最终英文投稿交付版/Full_Text_Reassessment_189.xlsx
+++ b/系统评价_最终英文投稿交付版/Full_Text_Reassessment_189.xlsx
@@ -1663,12 +1663,12 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>需核对纳入标准</t>
+          <t>倾向排除（作者暂定意见）</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>用户提供的全文进度表；未提供PDF文件、来源链接或具体待核对条款。保留为初评建议，最终状态待研究者确认。</t>
+          <t>作者于2026-10-27表示“倾向排除”。该意见为暂定倾向，尚非最终资格裁决；具体纳排依据及全文原文位置仍待核实。用户报告全文已获取，但PDF/来源链接未提供，当前工作区未核验。</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -1680,7 +1680,7 @@
       <c r="U12" s="2" t="n"/>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>PENDING_RESEARCHER_CONFIRMATION</t>
+          <t>PROVISIONAL_AUTHOR_LEAN_EXCLUDE_NOT_FINAL</t>
         </is>
       </c>
       <c r="W12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
sync final English manuscript and evidence files
</commit_message>
<xml_diff>
--- a/系统评价_最终英文投稿交付版/Full_Text_Reassessment_189.xlsx
+++ b/系统评价_最终英文投稿交付版/Full_Text_Reassessment_189.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="189篇逐项全文核查" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-10-28 aggregate update" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prior row-level snapshot" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'189篇逐项全文核查'!$A$1:$W$190</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Prior row-level snapshot'!$A$1:$W$190</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,6 +442,150 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Status category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Use in manuscript</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Abstract-level exclusion recommendations</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Aggregate update; record IDs unavailable</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Not counted as formal historical researcher exclusions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Completed full-text initial assessments</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Aggregate update</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>8 include recommendations; 4 exclude recommendations; 2 undecided</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Reports not obtained</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Aggregate update; record IDs unavailable</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Remain not retrieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>New inclusion candidates</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Incomplete extraction/appraisal</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Not incorporated into 35-study synthesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Completed synthesis</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>35 studies / 37 reports</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Existing verified workbooks</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Retained unchanged</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:W190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>